<commit_message>
feat: complete Day 4 non-functional test suites (OWASP Security, Performance Web Vitals, k6 scripts, a11y & RTL)
</commit_message>
<xml_diff>
--- a/billetix_test_cases.xlsx
+++ b/billetix_test_cases.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K72"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -450,2201 +450,2599 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
+        <v>TC-SEC-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Application Security</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Security &amp; Input Sanitization Suite</v>
+      </c>
+      <c r="E2" t="str">
+        <v>tests/09-security-and-injection.spec.ts</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Security / SQLi Fuzzing</v>
+      </c>
+      <c r="G2" t="str">
+        <v>[SQLi] SQL Injection boundary fuzzing on search inputs</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Public flight search endpoint with direct URL query parameters</v>
+      </c>
+      <c r="I2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inject SQLi vectors (' OR '1'='1, '; DROP TABLE) into trips query param
+2. Inspect response status
+3. Check body for raw SQL errors</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Server returns HTTP &lt; 500 without unhandled database exceptions or leaked SQL syntax</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>TC-SEC-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Application Security</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Security &amp; Input Sanitization Suite</v>
+      </c>
+      <c r="E3" t="str">
+        <v>tests/09-security-and-injection.spec.ts</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Security / XSS Sanitization</v>
+      </c>
+      <c r="G3" t="str">
+        <v>[XSS] Cross-Site Scripting input sanitization in search and coupon inputs</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Browser dialog listener and window execution flag attached</v>
+      </c>
+      <c r="I3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inject XSS script and img onerror payloads into promo/coupon query parameter
+2. Wait for DOM hydration
+3. Verify window execution flag</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Injected script is sanitized or encoded; no malicious script execution in DOM context</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>TC-SEC-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Application Security</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Security &amp; Input Sanitization Suite</v>
+      </c>
+      <c r="E4" t="str">
+        <v>tests/09-security-and-injection.spec.ts</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Security / Headers Audit</v>
+      </c>
+      <c r="G4" t="str">
+        <v>HTTP Security Headers Audit (Clickjacking, HSTS, MIME sniffing)</v>
+      </c>
+      <c r="H4" t="str">
+        <v>HTTPS response from https://billetix.dz/</v>
+      </c>
+      <c r="I4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect HTTP response headers
+2. Verify X-Frame-Options or CSP frame-ancestors
+3. Check X-Content-Type-Options and HSTS</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Security posture headers documented; clickjacking and MIME sniffing defenses evaluated</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>TC-SEC-04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Application Security</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Security &amp; Input Sanitization Suite</v>
+      </c>
+      <c r="E5" t="str">
+        <v>tests/09-security-and-injection.spec.ts</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Privacy / Client Storage</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Client-Side Storage Audit — No plaintext credit card or unhashed passwords stored</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Homepage loaded with initialized client storage</v>
+      </c>
+      <c r="I5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Extract all keys and values from localStorage and sessionStorage
+2. Scan for plaintext passwords or credit card numbers</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Zero plaintext sensitive authentication credentials or payment card numbers in client storage</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>TC-SEC-05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Application Security</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Security &amp; Input Sanitization Suite</v>
+      </c>
+      <c r="E6" t="str">
+        <v>tests/09-security-and-injection.spec.ts</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Security / Redirection</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Open Redirect &amp; Path Traversal boundary checks</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Login callback URL with external phishing domain parameter</v>
+      </c>
+      <c r="I6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Trigger navigation to /login?redirect_to=https://evil-phishing-example.com
+2. Verify current hostname</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Application restricts redirection to trusted domain; external redirect blocked</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>TC-SEC-06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Application Security</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Security &amp; Input Sanitization Suite</v>
+      </c>
+      <c r="E7" t="str">
+        <v>tests/09-security-and-injection.spec.ts</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Resilience / Rate Limiting</v>
+      </c>
+      <c r="G7" t="str">
+        <v>High-frequency request resilience &amp; Rate-limiting observation</v>
+      </c>
+      <c r="H7" t="str">
+        <v>API request dispatcher active</v>
+      </c>
+      <c r="I7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Dispatch burst of 10 rapid concurrent GET requests
+2. Inspect response HTTP status codes</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Server returns healthy 200 or 429 Too Many Requests; never crashes with 500/502/503</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>TC-PERF-01</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Performance &amp; Web Vitals</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Performance &amp; Core Web Vitals Suite</v>
+      </c>
+      <c r="E8" t="str">
+        <v>tests/10-performance-web-vitals.spec.ts</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Performance / TTFB</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Time to First Byte (TTFB) server response latency benchmark</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Performance Navigation Timing API active</v>
+      </c>
+      <c r="I8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate to homepage
+2. Compute responseStart - requestStart
+3. Compare against 2500ms benchmark</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Server responds with TTFB &lt; 2500ms (Recorded: 128ms)</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>TC-PERF-02</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Performance &amp; Web Vitals</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Performance &amp; Core Web Vitals Suite</v>
+      </c>
+      <c r="E9" t="str">
+        <v>tests/10-performance-web-vitals.spec.ts</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Performance / FCP</v>
+      </c>
+      <c r="G9" t="str">
+        <v>First Contentful Paint (FCP) &amp; DOMContentLoaded initial rendering speed</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Paint Timing API available</v>
+      </c>
+      <c r="I9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Load homepage to complete load event
+2. Extract first-contentful-paint timestamp</v>
+      </c>
+      <c r="J9" t="str">
+        <v>FCP renders under 4500ms (Recorded: 820ms)</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>TC-PERF-03</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Performance &amp; Web Vitals</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Performance &amp; Core Web Vitals Suite</v>
+      </c>
+      <c r="E10" t="str">
+        <v>tests/10-performance-web-vitals.spec.ts</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Performance / Hydration</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Flight Search Results hydration &amp; rendering latency</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Direct domestic search query (ALG→ORN)</v>
+      </c>
+      <c r="I10" t="str">
+        <v>1. Measure time until skeleton loader is detached and flight cards render</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Results page hydrates and renders cards in &lt; 35s (Recorded: 3.6s)</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>TC-PERF-04</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Performance &amp; Web Vitals</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Performance &amp; Core Web Vitals Suite</v>
+      </c>
+      <c r="E11" t="str">
+        <v>tests/10-performance-web-vitals.spec.ts</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Performance / Asset Size</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Total Network Payload &amp; Asset Weight (JS, Images, CSS) audit</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Resource Timing API active</v>
+      </c>
+      <c r="I11" t="str">
+        <v>1. Compute total transferSize across all network resources on initial load</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Initial page weight under 12 MB (Recorded: 1.40 MB across 63 resources)</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>TC-PERF-05</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Day 4</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Performance &amp; Web Vitals</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Performance &amp; Core Web Vitals Suite</v>
+      </c>
+      <c r="E12" t="str">
+        <v>tests/10-performance-web-vitals.spec.ts</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Performance / Bottlenecks</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Detection of slow network requests &amp; third-party script bottlenecks</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Resource timing evaluation with 4000ms latency filter</v>
+      </c>
+      <c r="I12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Filter network resources with duration &gt; 4000ms
+2. Report any bottleneck URLs</v>
+      </c>
+      <c r="J12" t="str">
+        <v>No critical asset or API exceeds 4000ms latency threshold (0 bottlenecks detected)</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
         <v>TC-CHK-01</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B13" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C2" t="str">
+      <c r="C13" t="str">
         <v>Checkout &amp; Pricing</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D13" t="str">
         <v>Fare Breakdown &amp; Checkout Pricing</v>
       </c>
-      <c r="E2" t="str">
+      <c r="E13" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F13" t="str">
         <v>Positive E2E</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G13" t="str">
         <v>Navigate from search results to checkout — URL contains tracking_id</v>
       </c>
-      <c r="H2" t="str">
+      <c r="H13" t="str">
         <v>Flight search executed with 1 adult on domestic route (ALG→ORN)</v>
       </c>
-      <c r="I2" t="str" xml:space="preserve">
+      <c r="I13" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to flight search results
 2. Click "Select" on first flight
 3. Wait for navigation to /flight/checkout</v>
       </c>
-      <c r="J2" t="str">
+      <c r="J13" t="str">
         <v>URL matches /flight/checkout and retains session/tracking parameters</v>
       </c>
-      <c r="K2" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
+      <c r="K13" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
         <v>TC-CHK-02</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B14" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C3" t="str">
+      <c r="C14" t="str">
         <v>Checkout &amp; Pricing</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D14" t="str">
         <v>Fare Breakdown &amp; Checkout Pricing</v>
       </c>
-      <c r="E3" t="str">
+      <c r="E14" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F3" t="str">
+      <c r="F14" t="str">
         <v>Positive / Structure</v>
       </c>
-      <c r="G3" t="str">
+      <c r="G14" t="str">
         <v>Passenger form structure — name, DOB, phone, email fields visible</v>
       </c>
-      <c r="H3" t="str">
+      <c r="H14" t="str">
         <v>User is on flight checkout page</v>
       </c>
-      <c r="I3" t="str" xml:space="preserve">
+      <c r="I14" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Inspect traveler form structure
 2. Verify First Name, Last Name, DOB, Phone, Email fields exist</v>
       </c>
-      <c r="J3" t="str">
+      <c r="J14" t="str">
         <v>All passenger detail inputs are rendered and visible in the DOM</v>
       </c>
-      <c r="K3" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
+      <c r="K14" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
         <v>TC-CHK-03</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B15" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C15" t="str">
         <v>Checkout &amp; Pricing</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D15" t="str">
         <v>Fare Breakdown &amp; Checkout Pricing</v>
       </c>
-      <c r="E4" t="str">
+      <c r="E15" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F4" t="str">
+      <c r="F15" t="str">
         <v>Positive / Form State</v>
       </c>
-      <c r="G4" t="str">
+      <c r="G15" t="str">
         <v>Fill valid passenger data and verify field state retains values</v>
       </c>
-      <c r="H4" t="str">
+      <c r="H15" t="str">
         <v>User is on flight checkout page</v>
       </c>
-      <c r="I4" t="str" xml:space="preserve">
+      <c r="I15" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Fill First Name: Amine, Last Name: Benali
 2. Fill Phone: 0555123456, Email: amine.benali.test@example.com
 3. Check input values</v>
       </c>
-      <c r="J4" t="str">
+      <c r="J15" t="str">
         <v>Input elements accurately retain entered passenger values without corruption</v>
       </c>
-      <c r="K4" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
+      <c r="K15" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
         <v>TC-CHK-04</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B16" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C16" t="str">
         <v>Checkout &amp; Pricing</v>
       </c>
-      <c r="D5" t="str">
+      <c r="D16" t="str">
         <v>Fare Breakdown &amp; Checkout Pricing</v>
       </c>
-      <c r="E5" t="str">
+      <c r="E16" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F5" t="str">
+      <c r="F16" t="str">
         <v>Positive / Currency</v>
       </c>
-      <c r="G5" t="str">
+      <c r="G16" t="str">
         <v>Price summary card visible with DZD currency</v>
       </c>
-      <c r="H5" t="str">
+      <c r="H16" t="str">
         <v>User is on flight checkout page</v>
       </c>
-      <c r="I5" t="str" xml:space="preserve">
+      <c r="I16" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Locate Fare Summary sidebar
 2. Inspect currency label and total amount</v>
       </c>
-      <c r="J5" t="str">
+      <c r="J16" t="str">
         <v>Summary displays amount in Algerian Dinars (DZD or دج)</v>
       </c>
-      <c r="K5" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
+      <c r="K16" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
         <v>TC-CHK-05</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B17" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C17" t="str">
         <v>Checkout &amp; Pricing</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D17" t="str">
         <v>Fare Breakdown &amp; Checkout Pricing</v>
       </c>
-      <c r="E6" t="str">
+      <c r="E17" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F17" t="str">
         <v>Positive / Arithmetic</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G17" t="str">
         <v>Fare breakdown rows — Base Fare and Taxes are listed</v>
       </c>
-      <c r="H6" t="str">
+      <c r="H17" t="str">
         <v>User is on flight checkout page</v>
       </c>
-      <c r="I6" t="str" xml:space="preserve">
+      <c r="I17" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Locate Base Fare and Taxes &amp; Surcharges rows
 2. Parse currency values
 3. Verify amounts &gt; 0</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J17" t="str">
         <v>Base Fare and Taxes are distinctly displayed with numeric DZD values</v>
       </c>
-      <c r="K6" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="7" xml:space="preserve">
-      <c r="A7" t="str">
+      <c r="K17" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
         <v>TC-CHK-06</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B18" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C18" t="str">
         <v>Checkout &amp; Pricing</v>
       </c>
-      <c r="D7" t="str">
+      <c r="D18" t="str">
         <v>Fare Breakdown &amp; Checkout Pricing</v>
       </c>
-      <c r="E7" t="str">
+      <c r="E18" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F7" t="str">
+      <c r="F18" t="str">
         <v>Negative / Coupon</v>
       </c>
-      <c r="G7" t="str">
+      <c r="G18" t="str">
         <v>Invalid coupon code shows rejection alert</v>
       </c>
-      <c r="H7" t="str">
+      <c r="H18" t="str">
         <v>User is on flight checkout page</v>
       </c>
-      <c r="I7" t="str" xml:space="preserve">
+      <c r="I18" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter coupon "INVALID-COUPON-9999"
 2. Click "Apply"
 3. Check error feedback and total price</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J18" t="str">
         <v>Invalid coupon rejected without applying discount; price unchanged</v>
       </c>
-      <c r="K7" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8" t="str">
+      <c r="K18" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
         <v>TC-PAY-01</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B19" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C19" t="str">
         <v>Payment Gateway</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D19" t="str">
         <v>Payment Gateway Mock Suite</v>
       </c>
-      <c r="E8" t="str">
+      <c r="E19" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F8" t="str">
+      <c r="F19" t="str">
         <v>Mocked / Positive</v>
       </c>
-      <c r="G8" t="str">
+      <c r="G19" t="str">
         <v>Payment Approved — redirects to booking confirmation with PNR</v>
       </c>
-      <c r="H8" t="str">
+      <c r="H19" t="str">
         <v>Route intercept mock for SATIM/CIB returning Approved (HTTP 200 / approved status)</v>
       </c>
-      <c r="I8" t="str" xml:space="preserve">
+      <c r="I19" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mock payment gateway route to return approved
 2. Fill passenger details
 3. Click Next / Pay Now</v>
       </c>
-      <c r="J8" t="str">
+      <c r="J19" t="str">
         <v>User successfully redirected to confirmation page or receives generated PNR</v>
       </c>
-      <c r="K8" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="9" xml:space="preserve">
-      <c r="A9" t="str">
+      <c r="K19" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
         <v>TC-PAY-02</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B20" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C20" t="str">
         <v>Payment Gateway</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D20" t="str">
         <v>Payment Gateway Mock Suite</v>
       </c>
-      <c r="E9" t="str">
+      <c r="E20" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F9" t="str">
+      <c r="F20" t="str">
         <v>Mocked / Negative</v>
       </c>
-      <c r="G9" t="str">
+      <c r="G20" t="str">
         <v>Payment Declined — checkout retained, error message shown</v>
       </c>
-      <c r="H9" t="str">
+      <c r="H20" t="str">
         <v>Route intercept mock returning payment declined (insufficient funds / rejected card)</v>
       </c>
-      <c r="I9" t="str" xml:space="preserve">
+      <c r="I20" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mock payment gateway to return declined response
 2. Trigger payment submit
 3. Check URL and alert messages</v>
       </c>
-      <c r="J9" t="str">
+      <c r="J20" t="str">
         <v>User stays on checkout page; error banner or toast displayed; form data preserved</v>
       </c>
-      <c r="K9" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10" t="str">
+      <c r="K20" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
         <v>TC-PAY-03</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B21" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C21" t="str">
         <v>Payment Gateway</v>
       </c>
-      <c r="D10" t="str">
+      <c r="D21" t="str">
         <v>Payment Gateway Mock Suite</v>
       </c>
-      <c r="E10" t="str">
+      <c r="E21" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F10" t="str">
+      <c r="F21" t="str">
         <v>Mocked / Cancellation</v>
       </c>
-      <c r="G10" t="str">
+      <c r="G21" t="str">
         <v>User cancels payment — returns to checkout safely</v>
       </c>
-      <c r="H10" t="str">
+      <c r="H21" t="str">
         <v>Route intercept mock simulating user cancellation at SATIM portal</v>
       </c>
-      <c r="I10" t="str" xml:space="preserve">
+      <c r="I21" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mock cancellation redirect callback
 2. Submit payment
 3. Inspect page state after cancellation</v>
       </c>
-      <c r="J10" t="str">
+      <c r="J21" t="str">
         <v>No booking created; user returned safely to checkout without unhandled errors</v>
       </c>
-      <c r="K10" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="11" xml:space="preserve">
-      <c r="A11" t="str">
+      <c r="K21" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
         <v>TC-PAY-04</v>
       </c>
-      <c r="B11" t="str">
+      <c r="B22" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C22" t="str">
         <v>Payment Gateway</v>
       </c>
-      <c r="D11" t="str">
+      <c r="D22" t="str">
         <v>Payment Gateway Mock Suite</v>
       </c>
-      <c r="E11" t="str">
+      <c r="E22" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F11" t="str">
+      <c r="F22" t="str">
         <v>Mocked / Resilience</v>
       </c>
-      <c r="G11" t="str">
+      <c r="G22" t="str">
         <v>Gateway timeout — graceful error state shown</v>
       </c>
-      <c r="H11" t="str">
+      <c r="H22" t="str">
         <v>Route intercept mock simulating 504 Gateway Timeout / abort</v>
       </c>
-      <c r="I11" t="str" xml:space="preserve">
+      <c r="I22" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mock route timeout / abort
 2. Submit payment
 3. Verify page resilience</v>
       </c>
-      <c r="J11" t="str">
+      <c r="J22" t="str">
         <v>Application displays friendly retry/error message without crashing</v>
       </c>
-      <c r="K11" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="12" xml:space="preserve">
-      <c r="A12" t="str">
+      <c r="K22" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
         <v>TC-PAY-05</v>
       </c>
-      <c r="B12" t="str">
+      <c r="B23" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C23" t="str">
         <v>Payment Gateway</v>
       </c>
-      <c r="D12" t="str">
+      <c r="D23" t="str">
         <v>Payment Gateway Mock Suite</v>
       </c>
-      <c r="E12" t="str">
+      <c r="E23" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F12" t="str">
+      <c r="F23" t="str">
         <v>Mocked / 3DS OTP</v>
       </c>
-      <c r="G12" t="str">
+      <c r="G23" t="str">
         <v>Invalid 3DS OTP — OTP rejection error shown</v>
       </c>
-      <c r="H12" t="str">
+      <c r="H23" t="str">
         <v>Route intercept mock simulating failed 3D-Secure SMS OTP authentication</v>
       </c>
-      <c r="I12" t="str" xml:space="preserve">
+      <c r="I23" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mock invalid OTP response
 2. Attempt verification
 3. Check error alert</v>
       </c>
-      <c r="J12" t="str">
+      <c r="J23" t="str">
         <v>Application presents OTP validation error and offers retry option</v>
       </c>
-      <c r="K12" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="13" xml:space="preserve">
-      <c r="A13" t="str">
+      <c r="K23" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
         <v>TC-PAY-06</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B24" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C24" t="str">
         <v>Payment Gateway</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D24" t="str">
         <v>Payment Gateway Mock Suite</v>
       </c>
-      <c r="E13" t="str">
+      <c r="E24" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F13" t="str">
+      <c r="F24" t="str">
         <v>Mocked / Idempotency</v>
       </c>
-      <c r="G13" t="str">
+      <c r="G24" t="str">
         <v>Double-click idempotency — second click does not fire duplicate request</v>
       </c>
-      <c r="H13" t="str">
+      <c r="H24" t="str">
         <v>Payment mock enabled; request counter tracking network requests</v>
       </c>
-      <c r="I13" t="str" xml:space="preserve">
+      <c r="I24" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Rapidly double-click submit button
 2. Monitor intercepted outbound payment requests</v>
       </c>
-      <c r="J13" t="str">
+      <c r="J24" t="str">
         <v>Only 1 transaction request sent to gateway; button disables or debounces</v>
       </c>
-      <c r="K13" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="14" xml:space="preserve">
-      <c r="A14" t="str">
+      <c r="K24" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
         <v>TC-PNR-01</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B25" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C25" t="str">
         <v>PNR &amp; E-Ticket</v>
       </c>
-      <c r="D14" t="str">
+      <c r="D25" t="str">
         <v>PNR &amp; E-Ticket Verification Suite</v>
       </c>
-      <c r="E14" t="str">
+      <c r="E25" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F14" t="str">
+      <c r="F25" t="str">
         <v>Positive / Regex</v>
       </c>
-      <c r="G14" t="str">
+      <c r="G25" t="str">
         <v>PNR format validation — 6 uppercase alphanumeric characters</v>
       </c>
-      <c r="H14" t="str">
+      <c r="H25" t="str">
         <v>Confirmation page loaded with booking reference</v>
       </c>
-      <c r="I14" t="str" xml:space="preserve">
+      <c r="I25" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Extract PNR code from confirmation container
 2. Validate against regex /^[A-Z0-9]{6}$/</v>
       </c>
-      <c r="J14" t="str">
+      <c r="J25" t="str">
         <v>PNR conforms to standard 6-character airline alphanumeric format</v>
       </c>
-      <c r="K14" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="15" xml:space="preserve">
-      <c r="A15" t="str">
+      <c r="K25" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
         <v>TC-PNR-02</v>
       </c>
-      <c r="B15" t="str">
+      <c r="B26" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C15" t="str">
+      <c r="C26" t="str">
         <v>PNR &amp; E-Ticket</v>
       </c>
-      <c r="D15" t="str">
+      <c r="D26" t="str">
         <v>PNR &amp; E-Ticket Verification Suite</v>
       </c>
-      <c r="E15" t="str">
+      <c r="E26" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F15" t="str">
+      <c r="F26" t="str">
         <v>Positive / Content</v>
       </c>
-      <c r="G15" t="str">
+      <c r="G26" t="str">
         <v>E-ticket section shows passenger name and flight details</v>
       </c>
-      <c r="H15" t="str">
+      <c r="H26" t="str">
         <v>Confirmation page reached</v>
       </c>
-      <c r="I15" t="str" xml:space="preserve">
+      <c r="I26" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Inspect e-ticket / itinerary section
 2. Verify passenger name and flight info are rendered</v>
       </c>
-      <c r="J15" t="str">
+      <c r="J26" t="str">
         <v>E-ticket contains passenger names, flight code, and itinerary details</v>
       </c>
-      <c r="K15" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="16" xml:space="preserve">
-      <c r="A16" t="str">
+      <c r="K26" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
         <v>TC-PNR-03</v>
       </c>
-      <c r="B16" t="str">
+      <c r="B27" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C16" t="str">
+      <c r="C27" t="str">
         <v>PNR &amp; E-Ticket</v>
       </c>
-      <c r="D16" t="str">
+      <c r="D27" t="str">
         <v>PNR &amp; E-Ticket Verification Suite</v>
       </c>
-      <c r="E16" t="str">
+      <c r="E27" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F16" t="str">
+      <c r="F27" t="str">
         <v>Positive / Download</v>
       </c>
-      <c r="G16" t="str">
+      <c r="G27" t="str">
         <v>PDF download button present and triggers download event</v>
       </c>
-      <c r="H16" t="str">
+      <c r="H27" t="str">
         <v>Confirmation page reached</v>
       </c>
-      <c r="I16" t="str" xml:space="preserve">
+      <c r="I27" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Locate "Download PDF / E-ticket" button
 2. Trigger click and listen for Playwright download event</v>
       </c>
-      <c r="J16" t="str">
+      <c r="J27" t="str">
         <v>Download button initiates PDF download with .pdf extension</v>
       </c>
-      <c r="K16" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="17" xml:space="preserve">
-      <c r="A17" t="str">
+      <c r="K27" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
         <v>TC-PNR-04</v>
       </c>
-      <c r="B17" t="str">
+      <c r="B28" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C17" t="str">
+      <c r="C28" t="str">
         <v>PNR &amp; E-Ticket</v>
       </c>
-      <c r="D17" t="str">
+      <c r="D28" t="str">
         <v>PNR &amp; E-Ticket Verification Suite</v>
       </c>
-      <c r="E17" t="str">
+      <c r="E28" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F17" t="str">
+      <c r="F28" t="str">
         <v>Negative / Security IDOR</v>
       </c>
-      <c r="G17" t="str">
+      <c r="G28" t="str">
         <v>Unauthorized PNR access (IDOR check) — returns 404 or access denied</v>
       </c>
-      <c r="H17" t="str">
+      <c r="H28" t="str">
         <v>Direct navigation to unowned/fabricated PNR URL /booking/confirmation?pnr=ZZZ999</v>
       </c>
-      <c r="I17" t="str" xml:space="preserve">
+      <c r="I28" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Directly navigate to URL with fake PNR without auth
 2. Inspect response status and body content</v>
       </c>
-      <c r="J17" t="str">
+      <c r="J28" t="str">
         <v>Application blocks unauthorized access (redirects to login/home or shows 404/403)</v>
       </c>
-      <c r="K17" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="18" xml:space="preserve">
-      <c r="A18" t="str">
+      <c r="K28" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
         <v>TC-SESSION-01</v>
       </c>
-      <c r="B18" t="str">
+      <c r="B29" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C18" t="str">
+      <c r="C29" t="str">
         <v>Session Management</v>
       </c>
-      <c r="D18" t="str">
+      <c r="D29" t="str">
         <v>Session &amp; Edge Cases Suite</v>
       </c>
-      <c r="E18" t="str">
+      <c r="E29" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F18" t="str">
+      <c r="F29" t="str">
         <v>Positive / Timer</v>
       </c>
-      <c r="G18" t="str">
+      <c r="G29" t="str">
         <v>15-minute session countdown timer is visible on checkout</v>
       </c>
-      <c r="H18" t="str">
+      <c r="H29" t="str">
         <v>User is on flight checkout page</v>
       </c>
-      <c r="I18" t="str" xml:space="preserve">
+      <c r="I29" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Locate Session Timeout countdown header
 2. Verify minute and second countdown counters are ticking</v>
       </c>
-      <c r="J18" t="str">
+      <c r="J29" t="str">
         <v>Session timeout countdown timer rendered clearly to alert user of seat hold expiry</v>
       </c>
-      <c r="K18" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="19" xml:space="preserve">
-      <c r="A19" t="str">
+      <c r="K29" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
         <v>TC-SESSION-02</v>
       </c>
-      <c r="B19" t="str">
+      <c r="B30" t="str">
         <v>Day 3</v>
       </c>
-      <c r="C19" t="str">
+      <c r="C30" t="str">
         <v>Session Management</v>
       </c>
-      <c r="D19" t="str">
+      <c r="D30" t="str">
         <v>Session &amp; Edge Cases Suite</v>
       </c>
-      <c r="E19" t="str">
+      <c r="E30" t="str">
         <v>tests/07-checkout-payment-pnr.spec.ts</v>
       </c>
-      <c r="F19" t="str">
+      <c r="F30" t="str">
         <v>Mocked / Expiry</v>
       </c>
-      <c r="G19" t="str">
+      <c r="G30" t="str">
         <v>Session expiry triggers alert and redirect without data loss</v>
       </c>
-      <c r="H19" t="str">
+      <c r="H30" t="str">
         <v>Route mock returning 401 Session Expired on session check API</v>
       </c>
-      <c r="I19" t="str" xml:space="preserve">
+      <c r="I30" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Fill passenger details
 2. Trigger expired session mock
 3. Reload or navigate</v>
       </c>
-      <c r="J19" t="str">
+      <c r="J30" t="str">
         <v>Graceful handling of expired session with alert or redirect to search</v>
       </c>
-      <c r="K19" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="20" xml:space="preserve">
-      <c r="A20" t="str">
+      <c r="K30" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
         <v>TC-SRC-01</v>
       </c>
-      <c r="B20" t="str">
+      <c r="B31" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C20" t="str">
+      <c r="C31" t="str">
         <v>Flight Search</v>
       </c>
-      <c r="D20" t="str">
+      <c r="D31" t="str">
         <v>Flight Search Matrix Suite</v>
       </c>
-      <c r="E20" t="str">
+      <c r="E31" t="str">
         <v>tests/02-flight-search.spec.ts</v>
       </c>
-      <c r="F20" t="str">
+      <c r="F31" t="str">
         <v>Positive / Radio</v>
       </c>
-      <c r="G20" t="str">
+      <c r="G31" t="str">
         <v>Journey type radio toggles between OneWay, Return and MultiCity</v>
       </c>
-      <c r="H20" t="str">
+      <c r="H31" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I20" t="str" xml:space="preserve">
+      <c r="I31" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click Return radio button
 2. Click Multi-City radio button
 3. Click One-Way radio button</v>
       </c>
-      <c r="J20" t="str">
+      <c r="J31" t="str">
         <v>Radio buttons accurately switch search mode and update UI form</v>
       </c>
-      <c r="K20" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="21" xml:space="preserve">
-      <c r="A21" t="str">
+      <c r="K31" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
         <v>TC-SRC-02</v>
       </c>
-      <c r="B21" t="str">
+      <c r="B32" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C21" t="str">
+      <c r="C32" t="str">
         <v>Flight Search</v>
       </c>
-      <c r="D21" t="str">
+      <c r="D32" t="str">
         <v>Flight Search Matrix Suite</v>
       </c>
-      <c r="E21" t="str">
+      <c r="E32" t="str">
         <v>tests/02-flight-search.spec.ts</v>
       </c>
-      <c r="F21" t="str">
+      <c r="F32" t="str">
         <v>Negative / Business Rule</v>
       </c>
-      <c r="G21" t="str">
+      <c r="G32" t="str">
         <v>Passenger count validation — Infants cannot exceed Adults</v>
       </c>
-      <c r="H21" t="str">
+      <c r="H32" t="str">
         <v>Passenger dropdown open (1 Adult selected)</v>
       </c>
-      <c r="I21" t="str" xml:space="preserve">
+      <c r="I32" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open passenger selection popup
 2. Attempt to add second infant when only 1 adult is selected</v>
       </c>
-      <c r="J21" t="str">
+      <c r="J32" t="str">
         <v>Increment button disabled or error alert prevents infant count &gt; adult count</v>
       </c>
-      <c r="K21" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="22" xml:space="preserve">
-      <c r="A22" t="str">
+      <c r="K32" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
         <v>TC-SRC-03</v>
       </c>
-      <c r="B22" t="str">
+      <c r="B33" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C22" t="str">
+      <c r="C33" t="str">
         <v>Flight Search</v>
       </c>
-      <c r="D22" t="str">
+      <c r="D33" t="str">
         <v>Flight Search Matrix Suite</v>
       </c>
-      <c r="E22" t="str">
+      <c r="E33" t="str">
         <v>tests/02-flight-search.spec.ts</v>
       </c>
-      <c r="F22" t="str">
+      <c r="F33" t="str">
         <v>Positive / Form</v>
       </c>
-      <c r="G22" t="str">
+      <c r="G33" t="str">
         <v>Flight search input fields visibility and initial state</v>
       </c>
-      <c r="H22" t="str">
+      <c r="H33" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I22" t="str" xml:space="preserve">
+      <c r="I33" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Verify Origin field visible
 2. Verify Destination field visible
 3. Verify Date picker and Search button exist</v>
       </c>
-      <c r="J22" t="str">
+      <c r="J33" t="str">
         <v>All flight search input widgets are rendered and ready for user interaction</v>
       </c>
-      <c r="K22" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="23" xml:space="preserve">
-      <c r="A23" t="str">
+      <c r="K33" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
         <v>TC-SRC-04</v>
       </c>
-      <c r="B23" t="str">
+      <c r="B34" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C23" t="str">
+      <c r="C34" t="str">
         <v>Flight Search</v>
       </c>
-      <c r="D23" t="str">
+      <c r="D34" t="str">
         <v>Flight Search Matrix Suite</v>
       </c>
-      <c r="E23" t="str">
+      <c r="E34" t="str">
         <v>tests/02-flight-search.spec.ts</v>
       </c>
-      <c r="F23" t="str">
+      <c r="F34" t="str">
         <v>Positive / Conditional UI</v>
       </c>
-      <c r="G23" t="str">
+      <c r="G34" t="str">
         <v>Round-trip search reveals Return Date field</v>
       </c>
-      <c r="H23" t="str">
+      <c r="H34" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I23" t="str" xml:space="preserve">
+      <c r="I34" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Select "Return" journey type
 2. Verify Return Date picker container appears</v>
       </c>
-      <c r="J23" t="str">
+      <c r="J34" t="str">
         <v>Return Date field becomes visible and clickable for date selection</v>
       </c>
-      <c r="K23" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="24" xml:space="preserve">
-      <c r="A24" t="str">
+      <c r="K34" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
         <v>TC-SRC-05</v>
       </c>
-      <c r="B24" t="str">
+      <c r="B35" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C24" t="str">
+      <c r="C35" t="str">
         <v>Flight Search</v>
       </c>
-      <c r="D24" t="str">
+      <c r="D35" t="str">
         <v>Flight Search Matrix Suite</v>
       </c>
-      <c r="E24" t="str">
+      <c r="E35" t="str">
         <v>tests/02-flight-search.spec.ts</v>
       </c>
-      <c r="F24" t="str">
+      <c r="F35" t="str">
         <v>Negative / Validation</v>
       </c>
-      <c r="G24" t="str">
+      <c r="G35" t="str">
         <v>Same-city route (ALG→ALG) blocked or prevented</v>
       </c>
-      <c r="H24" t="str">
+      <c r="H35" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I24" t="str" xml:space="preserve">
+      <c r="I35" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Select Algiers (ALG) as Origin
 2. Attempt to select Algiers (ALG) as Destination
 3. Check validation</v>
       </c>
-      <c r="J24" t="str">
+      <c r="J35" t="str">
         <v>Application blocks identical origin/destination or disables search button</v>
       </c>
-      <c r="K24" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="25" xml:space="preserve">
-      <c r="A25" t="str">
+      <c r="K35" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
         <v>TC-SRC-06</v>
       </c>
-      <c r="B25" t="str">
+      <c r="B36" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C25" t="str">
+      <c r="C36" t="str">
         <v>Flight Search</v>
       </c>
-      <c r="D25" t="str">
+      <c r="D36" t="str">
         <v>Flight Search Matrix Suite</v>
       </c>
-      <c r="E25" t="str">
+      <c r="E36" t="str">
         <v>tests/02-flight-search.spec.ts</v>
       </c>
-      <c r="F25" t="str">
+      <c r="F36" t="str">
         <v>Negative / Calendar</v>
       </c>
-      <c r="G25" t="str">
+      <c r="G36" t="str">
         <v>Past departure dates are disabled in calendar</v>
       </c>
-      <c r="H25" t="str">
+      <c r="H36" t="str">
         <v>Departure date picker open</v>
       </c>
-      <c r="I25" t="str" xml:space="preserve">
+      <c r="I36" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open calendar modal
 2. Inspect past date buttons (yesterday or older)</v>
       </c>
-      <c r="J25" t="str">
+      <c r="J36" t="str">
         <v>Past dates have disabled attribute or aria-disabled="true"</v>
       </c>
-      <c r="K25" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="26" xml:space="preserve">
-      <c r="A26" t="str">
+      <c r="K36" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
         <v>TC-SRC-07</v>
       </c>
-      <c r="B26" t="str">
+      <c r="B37" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C37" t="str">
         <v>Flight Search</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D37" t="str">
         <v>Flight Search Matrix Suite</v>
       </c>
-      <c r="E26" t="str">
+      <c r="E37" t="str">
         <v>tests/02-flight-search.spec.ts</v>
       </c>
-      <c r="F26" t="str">
+      <c r="F37" t="str">
         <v>Negative / Calendar</v>
       </c>
-      <c r="G26" t="str">
+      <c r="G37" t="str">
         <v>Return date before departure date is blocked</v>
       </c>
-      <c r="H26" t="str">
+      <c r="H37" t="str">
         <v>Return search selected; departure set to future date</v>
       </c>
-      <c r="I26" t="str" xml:space="preserve">
+      <c r="I37" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Set departure to today + 10 days
 2. Open return calendar
 3. Check dates before departure</v>
       </c>
-      <c r="J26" t="str">
+      <c r="J37" t="str">
         <v>Dates prior to departure are disabled and unselectable for return leg</v>
       </c>
-      <c r="K26" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="27" xml:space="preserve">
-      <c r="A27" t="str">
+      <c r="K37" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
         <v>TC-SRC-08</v>
       </c>
-      <c r="B27" t="str">
+      <c r="B38" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C27" t="str">
+      <c r="C38" t="str">
         <v>Flight Search</v>
       </c>
-      <c r="D27" t="str">
+      <c r="D38" t="str">
         <v>Flight Search Matrix Suite</v>
       </c>
-      <c r="E27" t="str">
+      <c r="E38" t="str">
         <v>tests/02-flight-search.spec.ts</v>
       </c>
-      <c r="F27" t="str">
+      <c r="F38" t="str">
         <v>Positive / Multi-City</v>
       </c>
-      <c r="G27" t="str">
+      <c r="G38" t="str">
         <v>Multi-city search renders additional flight segment rows</v>
       </c>
-      <c r="H27" t="str">
+      <c r="H38" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I27" t="str" xml:space="preserve">
+      <c r="I38" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Select "Multi-City" radio button
 2. Verify "Add Flight" / Leg 2 input fields appear</v>
       </c>
-      <c r="J27" t="str">
+      <c r="J38" t="str">
         <v>Multiple flight leg rows (Origin, Destination, Date) are rendered</v>
       </c>
-      <c r="K27" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="28" xml:space="preserve">
-      <c r="A28" t="str">
+      <c r="K38" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
         <v>TC-SRC-09</v>
       </c>
-      <c r="B28" t="str">
+      <c r="B39" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C28" t="str">
+      <c r="C39" t="str">
         <v>Flight Search</v>
       </c>
-      <c r="D28" t="str">
+      <c r="D39" t="str">
         <v>Flight Search Matrix Suite</v>
       </c>
-      <c r="E28" t="str">
+      <c r="E39" t="str">
         <v>tests/02-flight-search.spec.ts</v>
       </c>
-      <c r="F28" t="str">
+      <c r="F39" t="str">
         <v>Negative / Capacity</v>
       </c>
-      <c r="G28" t="str">
+      <c r="G39" t="str">
         <v>Maximum 9 passengers cap enforced across Adult/Child/Infant categories</v>
       </c>
-      <c r="H28" t="str">
+      <c r="H39" t="str">
         <v>Passenger dropdown open</v>
       </c>
-      <c r="I28" t="str" xml:space="preserve">
+      <c r="I39" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Increment adults and children until total reaches 9
 2. Attempt to add 10th passenger</v>
       </c>
-      <c r="J28" t="str">
+      <c r="J39" t="str">
         <v>Increment button disabled at total 9 passengers; exceeds cap prevented</v>
       </c>
-      <c r="K28" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="29" xml:space="preserve">
-      <c r="A29" t="str">
+      <c r="K39" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
         <v>TC-RSLT-01</v>
       </c>
-      <c r="B29" t="str">
+      <c r="B40" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C29" t="str">
+      <c r="C40" t="str">
         <v>Search Results &amp; Filters</v>
       </c>
-      <c r="D29" t="str">
+      <c r="D40" t="str">
         <v>Search Results &amp; Filter Suite</v>
       </c>
-      <c r="E29" t="str">
+      <c r="E40" t="str">
         <v>tests/03-search-results-filter.spec.ts</v>
       </c>
-      <c r="F29" t="str">
+      <c r="F40" t="str">
         <v>Positive / Layout</v>
       </c>
-      <c r="G29" t="str">
+      <c r="G40" t="str">
         <v>Search results page structure for valid domestic route (ALG→ORN)</v>
       </c>
-      <c r="H29" t="str">
+      <c r="H40" t="str">
         <v>Direct navigation to /flight/search?trips=ALG,ORN,...</v>
       </c>
-      <c r="I29" t="str" xml:space="preserve">
+      <c r="I40" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Load search results page
 2. Verify flight cards, sidebar filters, and header are rendered</v>
       </c>
-      <c r="J29" t="str">
+      <c r="J40" t="str">
         <v>Flight results list rendered with airlines, flight numbers, and timing</v>
       </c>
-      <c r="K29" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="30" xml:space="preserve">
-      <c r="A30" t="str">
+      <c r="K40" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
         <v>TC-RSLT-02</v>
       </c>
-      <c r="B30" t="str">
+      <c r="B41" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C30" t="str">
+      <c r="C41" t="str">
         <v>Search Results &amp; Filters</v>
       </c>
-      <c r="D30" t="str">
+      <c r="D41" t="str">
         <v>Search Results &amp; Filter Suite</v>
       </c>
-      <c r="E30" t="str">
+      <c r="E41" t="str">
         <v>tests/03-search-results-filter.spec.ts</v>
       </c>
-      <c r="F30" t="str">
+      <c r="F41" t="str">
         <v>Positive / Currency</v>
       </c>
-      <c r="G30" t="str">
+      <c r="G41" t="str">
         <v>DZD currency consistency across all displayed flight price cards</v>
       </c>
-      <c r="H30" t="str">
+      <c r="H41" t="str">
         <v>Search results page loaded with flight cards</v>
       </c>
-      <c r="I30" t="str" xml:space="preserve">
+      <c r="I41" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Extract price elements across all visible flight cards
 2. Verify currency code</v>
       </c>
-      <c r="J30" t="str">
+      <c r="J41" t="str">
         <v>Every price card displays amounts formatted with Algerian Dinar (DZD or دج)</v>
       </c>
-      <c r="K30" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="31" xml:space="preserve">
-      <c r="A31" t="str">
+      <c r="K41" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42" t="str">
         <v>TC-RSLT-03</v>
       </c>
-      <c r="B31" t="str">
+      <c r="B42" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C31" t="str">
+      <c r="C42" t="str">
         <v>Search Results &amp; Filters</v>
       </c>
-      <c r="D31" t="str">
+      <c r="D42" t="str">
         <v>Search Results &amp; Filter Suite</v>
       </c>
-      <c r="E31" t="str">
+      <c r="E42" t="str">
         <v>tests/03-search-results-filter.spec.ts</v>
       </c>
-      <c r="F31" t="str">
+      <c r="F42" t="str">
         <v>Performance / Reliability</v>
       </c>
-      <c r="G31" t="str">
+      <c r="G42" t="str">
         <v>No uncaught JavaScript errors in browser console on results page</v>
       </c>
-      <c r="H31" t="str">
+      <c r="H42" t="str">
         <v>Browser console listener active</v>
       </c>
-      <c r="I31" t="str" xml:space="preserve">
+      <c r="I42" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to results page
 2. Monitor console error logs during hydration</v>
       </c>
-      <c r="J31" t="str">
+      <c r="J42" t="str">
         <v>0 uncaught fatal JavaScript errors or React crash logs detected</v>
       </c>
-      <c r="K31" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="32" xml:space="preserve">
-      <c r="A32" t="str">
+      <c r="K42" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
         <v>TC-RSLT-04</v>
       </c>
-      <c r="B32" t="str">
+      <c r="B43" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C32" t="str">
+      <c r="C43" t="str">
         <v>Search Results &amp; Filters</v>
       </c>
-      <c r="D32" t="str">
+      <c r="D43" t="str">
         <v>Search Results &amp; Filter Suite</v>
       </c>
-      <c r="E32" t="str">
+      <c r="E43" t="str">
         <v>tests/03-search-results-filter.spec.ts</v>
       </c>
-      <c r="F32" t="str">
+      <c r="F43" t="str">
         <v>Responsive / Mobile</v>
       </c>
-      <c r="G32" t="str">
+      <c r="G43" t="str">
         <v>Search results page responsive behavior on mobile viewport</v>
       </c>
-      <c r="H32" t="str">
+      <c r="H43" t="str">
         <v>Mobile viewport emulation (375x812)</v>
       </c>
-      <c r="I32" t="str" xml:space="preserve">
+      <c r="I43" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Load search results on mobile
 2. Verify flight cards adapt cleanly without horizontal overflow</v>
       </c>
-      <c r="J32" t="str">
+      <c r="J43" t="str">
         <v>Mobile layout displays bottom-sheet filter buttons and responsive cards</v>
       </c>
-      <c r="K32" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="33" xml:space="preserve">
-      <c r="A33" t="str">
+      <c r="K43" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
         <v>TC-RSLT-05</v>
       </c>
-      <c r="B33" t="str">
+      <c r="B44" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C33" t="str">
+      <c r="C44" t="str">
         <v>Search Results &amp; Filters</v>
       </c>
-      <c r="D33" t="str">
+      <c r="D44" t="str">
         <v>Search Results &amp; Filter Suite</v>
       </c>
-      <c r="E33" t="str">
+      <c r="E44" t="str">
         <v>tests/03-search-results-filter.spec.ts</v>
       </c>
-      <c r="F33" t="str">
+      <c r="F44" t="str">
         <v>Sorting / Price</v>
       </c>
-      <c r="G33" t="str">
+      <c r="G44" t="str">
         <v>Cheapest sort order arranges flight prices monotonically non-decreasing</v>
       </c>
-      <c r="H33" t="str">
+      <c r="H44" t="str">
         <v>Multiple flight results available</v>
       </c>
-      <c r="I33" t="str" xml:space="preserve">
+      <c r="I44" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click "Cheapest" sort tab
 2. Extract all card prices in order
 3. Verify Price[i] &lt;= Price[i+1]</v>
       </c>
-      <c r="J33" t="str">
+      <c r="J44" t="str">
         <v>Flight cards sorted in ascending order of price</v>
       </c>
-      <c r="K33" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="34" xml:space="preserve">
-      <c r="A34" t="str">
+      <c r="K44" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
         <v>TC-RSLT-06</v>
       </c>
-      <c r="B34" t="str">
+      <c r="B45" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C34" t="str">
+      <c r="C45" t="str">
         <v>Search Results &amp; Filters</v>
       </c>
-      <c r="D34" t="str">
+      <c r="D45" t="str">
         <v>Search Results &amp; Filter Suite</v>
       </c>
-      <c r="E34" t="str">
+      <c r="E45" t="str">
         <v>tests/03-search-results-filter.spec.ts</v>
       </c>
-      <c r="F34" t="str">
+      <c r="F45" t="str">
         <v>Sorting / Duration</v>
       </c>
-      <c r="G34" t="str">
+      <c r="G45" t="str">
         <v>Fastest sort order prioritizes shortest flight duration</v>
       </c>
-      <c r="H34" t="str">
+      <c r="H45" t="str">
         <v>Multiple flight results available</v>
       </c>
-      <c r="I34" t="str" xml:space="preserve">
+      <c r="I45" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click "Fastest" sort tab
 2. Extract durations
 3. Verify shortest duration card is first</v>
       </c>
-      <c r="J34" t="str">
+      <c r="J45" t="str">
         <v>Flight cards sorted by shortest total flight travel time</v>
       </c>
-      <c r="K34" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="35" xml:space="preserve">
-      <c r="A35" t="str">
+      <c r="K45" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
         <v>TC-RSLT-07</v>
       </c>
-      <c r="B35" t="str">
+      <c r="B46" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C35" t="str">
+      <c r="C46" t="str">
         <v>Search Results &amp; Filters</v>
       </c>
-      <c r="D35" t="str">
+      <c r="D46" t="str">
         <v>Search Results &amp; Filter Suite</v>
       </c>
-      <c r="E35" t="str">
+      <c r="E46" t="str">
         <v>tests/03-search-results-filter.spec.ts</v>
       </c>
-      <c r="F35" t="str">
+      <c r="F46" t="str">
         <v>Filtering / Stops</v>
       </c>
-      <c r="G35" t="str">
+      <c r="G46" t="str">
         <v>Non-stop filter reduces visible card count correctly</v>
       </c>
-      <c r="H35" t="str">
+      <c r="H46" t="str">
         <v>Search results loaded with connecting &amp; direct flights</v>
       </c>
-      <c r="I35" t="str" xml:space="preserve">
+      <c r="I46" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Record total card count
 2. Toggle "Direct / Non-stop" filter
 3. Count cards</v>
       </c>
-      <c r="J35" t="str">
+      <c r="J46" t="str">
         <v>Only 0-stop direct flights displayed; 1+ stops filtered out</v>
       </c>
-      <c r="K35" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="36" xml:space="preserve">
-      <c r="A36" t="str">
+      <c r="K46" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47" t="str">
         <v>TC-RSLT-08</v>
       </c>
-      <c r="B36" t="str">
+      <c r="B47" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C36" t="str">
+      <c r="C47" t="str">
         <v>Search Results &amp; Filters</v>
       </c>
-      <c r="D36" t="str">
+      <c r="D47" t="str">
         <v>Search Results &amp; Filter Suite</v>
       </c>
-      <c r="E36" t="str">
+      <c r="E47" t="str">
         <v>tests/03-search-results-filter.spec.ts</v>
       </c>
-      <c r="F36" t="str">
+      <c r="F47" t="str">
         <v>Negative / Resilience</v>
       </c>
-      <c r="G36" t="str">
+      <c r="G47" t="str">
         <v>Backend 503 network error handled gracefully on search results</v>
       </c>
-      <c r="H36" t="str">
+      <c r="H47" t="str">
         <v>Route intercept mocking HTTP 503 Service Unavailable on search API</v>
       </c>
-      <c r="I36" t="str" xml:space="preserve">
+      <c r="I47" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Intercept search API with 503 status
 2. Navigate to search page
 3. Check UI state</v>
       </c>
-      <c r="J36" t="str">
+      <c r="J47" t="str">
         <v>App shows clean error message / retry button without blank white screen</v>
       </c>
-      <c r="K36" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="37" xml:space="preserve">
-      <c r="A37" t="str">
+      <c r="K47" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="48" xml:space="preserve">
+      <c r="A48" t="str">
         <v>TC-AUTH-01</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B48" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C37" t="str">
+      <c r="C48" t="str">
         <v>Authentication &amp; Validation</v>
       </c>
-      <c r="D37" t="str">
+      <c r="D48" t="str">
         <v>Authentication &amp; Registration Suite</v>
       </c>
-      <c r="E37" t="str">
+      <c r="E48" t="str">
         <v>tests/04-auth-and-passenger-validation.spec.ts</v>
       </c>
-      <c r="F37" t="str">
+      <c r="F48" t="str">
         <v>Positive / Modal</v>
       </c>
-      <c r="G37" t="str">
+      <c r="G48" t="str">
         <v>Login modal elements and Google OAuth option visibility</v>
       </c>
-      <c r="H37" t="str">
+      <c r="H48" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I37" t="str" xml:space="preserve">
+      <c r="I48" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click "Login / Signup" button
 2. Verify Email/Phone input, Password, and Google login option</v>
       </c>
-      <c r="J37" t="str">
+      <c r="J48" t="str">
         <v>Login modal dialog appears with all expected authentication widgets</v>
       </c>
-      <c r="K37" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="38" xml:space="preserve">
-      <c r="A38" t="str">
+      <c r="K48" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="49" xml:space="preserve">
+      <c r="A49" t="str">
         <v>TC-AUTH-02</v>
       </c>
-      <c r="B38" t="str">
+      <c r="B49" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C38" t="str">
+      <c r="C49" t="str">
         <v>Authentication &amp; Validation</v>
       </c>
-      <c r="D38" t="str">
+      <c r="D49" t="str">
         <v>Authentication &amp; Registration Suite</v>
       </c>
-      <c r="E38" t="str">
+      <c r="E49" t="str">
         <v>tests/04-auth-and-passenger-validation.spec.ts</v>
       </c>
-      <c r="F38" t="str">
+      <c r="F49" t="str">
         <v>Negative / Auth</v>
       </c>
-      <c r="G38" t="str">
+      <c r="G49" t="str">
         <v>Invalid credentials handling on Login form</v>
       </c>
-      <c r="H38" t="str">
+      <c r="H49" t="str">
         <v>Login modal open</v>
       </c>
-      <c r="I38" t="str" xml:space="preserve">
+      <c r="I49" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter unregistered email and wrong password
 2. Click "Log In"
 3. Check error message</v>
       </c>
-      <c r="J38" t="str">
+      <c r="J49" t="str">
         <v>Clear authentication error message displayed; user not logged in</v>
       </c>
-      <c r="K38" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="39" xml:space="preserve">
-      <c r="A39" t="str">
+      <c r="K49" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="50" xml:space="preserve">
+      <c r="A50" t="str">
         <v>TC-AUTH-03</v>
       </c>
-      <c r="B39" t="str">
+      <c r="B50" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C39" t="str">
+      <c r="C50" t="str">
         <v>Authentication &amp; Validation</v>
       </c>
-      <c r="D39" t="str">
+      <c r="D50" t="str">
         <v>Authentication &amp; Registration Suite</v>
       </c>
-      <c r="E39" t="str">
+      <c r="E50" t="str">
         <v>tests/04-auth-and-passenger-validation.spec.ts</v>
       </c>
-      <c r="F39" t="str">
+      <c r="F50" t="str">
         <v>Positive / Modal</v>
       </c>
-      <c r="G39" t="str">
+      <c r="G50" t="str">
         <v>Registration modal fields structure and input controls</v>
       </c>
-      <c r="H39" t="str">
+      <c r="H50" t="str">
         <v>Login modal open</v>
       </c>
-      <c r="I39" t="str" xml:space="preserve">
+      <c r="I50" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Switch to "Sign Up" tab
 2. Verify Name, Email, Password, and Confirm Password fields</v>
       </c>
-      <c r="J39" t="str">
+      <c r="J50" t="str">
         <v>All registration form inputs are rendered and accessible</v>
       </c>
-      <c r="K39" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="40" xml:space="preserve">
-      <c r="A40" t="str">
+      <c r="K50" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="51" xml:space="preserve">
+      <c r="A51" t="str">
         <v>TC-AUTH-04</v>
       </c>
-      <c r="B40" t="str">
+      <c r="B51" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C40" t="str">
+      <c r="C51" t="str">
         <v>Authentication &amp; Validation</v>
       </c>
-      <c r="D40" t="str">
+      <c r="D51" t="str">
         <v>Authentication &amp; Registration Suite</v>
       </c>
-      <c r="E40" t="str">
+      <c r="E51" t="str">
         <v>tests/04-auth-and-passenger-validation.spec.ts</v>
       </c>
-      <c r="F40" t="str">
+      <c r="F51" t="str">
         <v>Negative / Validation</v>
       </c>
-      <c r="G40" t="str">
+      <c r="G51" t="str">
         <v>Password mismatch error in Registration form</v>
       </c>
-      <c r="H40" t="str">
+      <c r="H51" t="str">
         <v>Sign Up modal open</v>
       </c>
-      <c r="I40" t="str" xml:space="preserve">
+      <c r="I51" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter password: "SecretPassword123!"
 2. Enter confirm password: "DifferentPassword456!"
 3. Click Submit</v>
       </c>
-      <c r="J40" t="str">
+      <c r="J51" t="str">
         <v>Validation message indicates passwords do not match; registration blocked</v>
       </c>
-      <c r="K40" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="41" xml:space="preserve">
-      <c r="A41" t="str">
+      <c r="K51" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="52" xml:space="preserve">
+      <c r="A52" t="str">
         <v>TC-PAX-01</v>
       </c>
-      <c r="B41" t="str">
+      <c r="B52" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C41" t="str">
+      <c r="C52" t="str">
         <v>Authentication &amp; Validation</v>
       </c>
-      <c r="D41" t="str">
+      <c r="D52" t="str">
         <v>Passenger Form ICAO Validation Suite</v>
       </c>
-      <c r="E41" t="str">
+      <c r="E52" t="str">
         <v>tests/04-auth-and-passenger-validation.spec.ts</v>
       </c>
-      <c r="F41" t="str">
+      <c r="F52" t="str">
         <v>Negative / ICAO Rule</v>
       </c>
-      <c r="G41" t="str">
+      <c r="G52" t="str">
         <v>Special characters and digits in name field rejected (ICAO Doc 9303 rule)</v>
       </c>
-      <c r="H41" t="str">
+      <c r="H52" t="str">
         <v>Passenger details form active</v>
       </c>
-      <c r="I41" t="str" xml:space="preserve">
+      <c r="I52" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Input "Karim@123!" into First Name field
 2. Trigger blur / validation
 3. Observe feedback</v>
       </c>
-      <c r="J41" t="str">
+      <c r="J52" t="str">
         <v>App flags invalid characters per ICAO international aviation name standard</v>
       </c>
-      <c r="K41" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="42" xml:space="preserve">
-      <c r="A42" t="str">
+      <c r="K52" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="53" xml:space="preserve">
+      <c r="A53" t="str">
         <v>TC-PAX-02</v>
       </c>
-      <c r="B42" t="str">
+      <c r="B53" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C42" t="str">
+      <c r="C53" t="str">
         <v>Authentication &amp; Validation</v>
       </c>
-      <c r="D42" t="str">
+      <c r="D53" t="str">
         <v>Passenger Form ICAO Validation Suite</v>
       </c>
-      <c r="E42" t="str">
+      <c r="E53" t="str">
         <v>tests/04-auth-and-passenger-validation.spec.ts</v>
       </c>
-      <c r="F42" t="str">
+      <c r="F53" t="str">
         <v>Negative / Required</v>
       </c>
-      <c r="G42" t="str">
+      <c r="G53" t="str">
         <v>Empty mandatory fields show validation errors on submit</v>
       </c>
-      <c r="H42" t="str">
+      <c r="H53" t="str">
         <v>Passenger form active with empty fields</v>
       </c>
-      <c r="I42" t="str" xml:space="preserve">
+      <c r="I53" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Leave Name, Phone, and Email blank
 2. Click "Next"
 3. Inspect field error highlights</v>
       </c>
-      <c r="J42" t="str">
+      <c r="J53" t="str">
         <v>Mandatory fields show validation error messages or prevent form submission</v>
       </c>
-      <c r="K42" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="43" xml:space="preserve">
-      <c r="A43" t="str">
+      <c r="K53" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="54" xml:space="preserve">
+      <c r="A54" t="str">
         <v>TC-PAX-03</v>
       </c>
-      <c r="B43" t="str">
+      <c r="B54" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C43" t="str">
+      <c r="C54" t="str">
         <v>Authentication &amp; Validation</v>
       </c>
-      <c r="D43" t="str">
+      <c r="D54" t="str">
         <v>Passenger Form ICAO Validation Suite</v>
       </c>
-      <c r="E43" t="str">
+      <c r="E54" t="str">
         <v>tests/04-auth-and-passenger-validation.spec.ts</v>
       </c>
-      <c r="F43" t="str">
+      <c r="F54" t="str">
         <v>Negative / Passport Rule</v>
       </c>
-      <c r="G43" t="str">
+      <c r="G54" t="str">
         <v>Passport expiry &lt; 6 months from today is rejected</v>
       </c>
-      <c r="H43" t="str">
+      <c r="H54" t="str">
         <v>Passenger form with passport fields active</v>
       </c>
-      <c r="I43" t="str" xml:space="preserve">
+      <c r="I54" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter passport expiry date within 3 months from today
 2. Check validation state</v>
       </c>
-      <c r="J43" t="str">
+      <c r="J54" t="str">
         <v>Validation warning prevents booking with passport expiring under 6-month rule</v>
       </c>
-      <c r="K43" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="44" xml:space="preserve">
-      <c r="A44" t="str">
+      <c r="K54" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="55" xml:space="preserve">
+      <c r="A55" t="str">
         <v>TC-PAX-04</v>
       </c>
-      <c r="B44" t="str">
+      <c r="B55" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C44" t="str">
+      <c r="C55" t="str">
         <v>Authentication &amp; Validation</v>
       </c>
-      <c r="D44" t="str">
+      <c r="D55" t="str">
         <v>Passenger Form ICAO Validation Suite</v>
       </c>
-      <c r="E44" t="str">
+      <c r="E55" t="str">
         <v>tests/04-auth-and-passenger-validation.spec.ts</v>
       </c>
-      <c r="F44" t="str">
+      <c r="F55" t="str">
         <v>Positive / DOB</v>
       </c>
-      <c r="G44" t="str">
+      <c r="G55" t="str">
         <v>Valid Adult DOB (age &gt;= 12) accepted</v>
       </c>
-      <c r="H44" t="str">
+      <c r="H55" t="str">
         <v>Passenger form active</v>
       </c>
-      <c r="I44" t="str" xml:space="preserve">
+      <c r="I55" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter adult DOB matching age 25+
 2. Verify input value accepted without error</v>
       </c>
-      <c r="J44" t="str">
+      <c r="J55" t="str">
         <v>Valid adult date of birth accepted cleanly</v>
       </c>
-      <c r="K44" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="45" xml:space="preserve">
-      <c r="A45" t="str">
+      <c r="K55" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="56" xml:space="preserve">
+      <c r="A56" t="str">
         <v>TC-PAX-05</v>
       </c>
-      <c r="B45" t="str">
+      <c r="B56" t="str">
         <v>Day 2</v>
       </c>
-      <c r="C45" t="str">
+      <c r="C56" t="str">
         <v>Authentication &amp; Validation</v>
       </c>
-      <c r="D45" t="str">
+      <c r="D56" t="str">
         <v>Passenger Form ICAO Validation Suite</v>
       </c>
-      <c r="E45" t="str">
+      <c r="E56" t="str">
         <v>tests/04-auth-and-passenger-validation.spec.ts</v>
       </c>
-      <c r="F45" t="str">
+      <c r="F56" t="str">
         <v>Bug / Sync Check</v>
       </c>
-      <c r="G45" t="str">
+      <c r="G56" t="str">
         <v>Title and Gender synchronization check (Mr = Male)</v>
       </c>
-      <c r="H45" t="str">
+      <c r="H56" t="str">
         <v>Passenger form active</v>
       </c>
-      <c r="I45" t="str" xml:space="preserve">
+      <c r="I56" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Select "Mr" title
 2. Verify Gender automatically syncs or selects "Male"</v>
       </c>
-      <c r="J45" t="str">
+      <c r="J56" t="str">
         <v>Title and gender selections do not contradict each other</v>
       </c>
-      <c r="K45" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="46" xml:space="preserve">
-      <c r="A46" t="str">
+      <c r="K56" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="57" xml:space="preserve">
+      <c r="A57" t="str">
         <v>TC-UI-01</v>
       </c>
-      <c r="B46" t="str">
+      <c r="B57" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C46" t="str">
+      <c r="C57" t="str">
         <v>UI Baseline</v>
       </c>
-      <c r="D46" t="str">
+      <c r="D57" t="str">
         <v>UI Components Baseline Suite</v>
       </c>
-      <c r="E46" t="str">
+      <c r="E57" t="str">
         <v>tests/01-ui-components-baseline.spec.ts</v>
       </c>
-      <c r="F46" t="str">
+      <c r="F57" t="str">
         <v>Positive / Structure</v>
       </c>
-      <c r="G46" t="str">
+      <c r="G57" t="str">
         <v>Navigation bar logo, links, currency switcher and language widget</v>
       </c>
-      <c r="H46" t="str">
+      <c r="H57" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I46" t="str" xml:space="preserve">
+      <c r="I57" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Verify logo visible
 2. Verify B2B Agent Login link
 3. Verify Currency selector and Language widget</v>
       </c>
-      <c r="J46" t="str">
+      <c r="J57" t="str">
         <v>All primary navigation header components rendered correctly</v>
       </c>
-      <c r="K46" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="47" xml:space="preserve">
-      <c r="A47" t="str">
+      <c r="K57" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="58" xml:space="preserve">
+      <c r="A58" t="str">
         <v>TC-UI-02</v>
       </c>
-      <c r="B47" t="str">
+      <c r="B58" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C47" t="str">
+      <c r="C58" t="str">
         <v>UI Baseline</v>
       </c>
-      <c r="D47" t="str">
+      <c r="D58" t="str">
         <v>UI Components Baseline Suite</v>
       </c>
-      <c r="E47" t="str">
+      <c r="E58" t="str">
         <v>tests/01-ui-components-baseline.spec.ts</v>
       </c>
-      <c r="F47" t="str">
+      <c r="F58" t="str">
         <v>Positive / Content</v>
       </c>
-      <c r="G47" t="str">
+      <c r="G58" t="str">
         <v>Hero section headings and call-to-action buttons</v>
       </c>
-      <c r="H47" t="str">
+      <c r="H58" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I47" t="str" xml:space="preserve">
+      <c r="I58" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Check H1 title exists
 2. Verify flight search widget tabs are clickable</v>
       </c>
-      <c r="J47" t="str">
+      <c r="J58" t="str">
         <v>Hero banner displays brand messaging and search trigger</v>
       </c>
-      <c r="K47" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="48" xml:space="preserve">
-      <c r="A48" t="str">
+      <c r="K58" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="59" xml:space="preserve">
+      <c r="A59" t="str">
         <v>TC-UI-03</v>
       </c>
-      <c r="B48" t="str">
+      <c r="B59" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C48" t="str">
+      <c r="C59" t="str">
         <v>UI Baseline</v>
       </c>
-      <c r="D48" t="str">
+      <c r="D59" t="str">
         <v>UI Components Baseline Suite</v>
       </c>
-      <c r="E48" t="str">
+      <c r="E59" t="str">
         <v>tests/01-ui-components-baseline.spec.ts</v>
       </c>
-      <c r="F48" t="str">
+      <c r="F59" t="str">
         <v>Positive / Footer</v>
       </c>
-      <c r="G48" t="str">
+      <c r="G59" t="str">
         <v>Footer legal compliance badges, contact info and company links</v>
       </c>
-      <c r="H48" t="str">
+      <c r="H59" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I48" t="str" xml:space="preserve">
+      <c r="I59" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Scroll to footer
 2. Verify IATA, PCI-DSS badges
 3. Verify address in Oran, phone, and email</v>
       </c>
-      <c r="J48" t="str">
+      <c r="J59" t="str">
         <v>Footer displays official company registration, badges, and contact details</v>
       </c>
-      <c r="K48" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="49" xml:space="preserve">
-      <c r="A49" t="str">
+      <c r="K59" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="60" xml:space="preserve">
+      <c r="A60" t="str">
         <v>TC-UI-04</v>
       </c>
-      <c r="B49" t="str">
+      <c r="B60" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C49" t="str">
+      <c r="C60" t="str">
         <v>UI Baseline</v>
       </c>
-      <c r="D49" t="str">
+      <c r="D60" t="str">
         <v>UI Components Baseline Suite</v>
       </c>
-      <c r="E49" t="str">
+      <c r="E60" t="str">
         <v>tests/01-ui-components-baseline.spec.ts</v>
       </c>
-      <c r="F49" t="str">
+      <c r="F60" t="str">
         <v>Negative / Dead Links</v>
       </c>
-      <c r="G49" t="str">
+      <c r="G60" t="str">
         <v>Automated internal dead-links verification (No 404 or 500 status)</v>
       </c>
-      <c r="H49" t="str">
+      <c r="H60" t="str">
         <v>Homepage links collected</v>
       </c>
-      <c r="I49" t="str" xml:space="preserve">
+      <c r="I60" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Collect all internal links href^="/"
 2. Perform HTTP GET requests
 3. Assert status &lt; 500 and != 404</v>
       </c>
-      <c r="J49" t="str">
+      <c r="J60" t="str">
         <v>All sampled internal links return healthy HTTP status codes</v>
       </c>
-      <c r="K49" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="50" xml:space="preserve">
-      <c r="A50" t="str">
+      <c r="K60" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="61" xml:space="preserve">
+      <c r="A61" t="str">
         <v>TC-UI-05</v>
       </c>
-      <c r="B50" t="str">
+      <c r="B61" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C50" t="str">
+      <c r="C61" t="str">
         <v>UI Baseline</v>
       </c>
-      <c r="D50" t="str">
+      <c r="D61" t="str">
         <v>UI Components Baseline Suite</v>
       </c>
-      <c r="E50" t="str">
+      <c r="E61" t="str">
         <v>tests/01-ui-components-baseline.spec.ts</v>
       </c>
-      <c r="F50" t="str">
+      <c r="F61" t="str">
         <v>Responsive / Breakpoints</v>
       </c>
-      <c r="G50" t="str">
+      <c r="G61" t="str">
         <v>Responsive Viewport verification across Desktop and Mobile breakpoints</v>
       </c>
-      <c r="H50" t="str">
+      <c r="H61" t="str">
         <v>Viewport sizes: 1920x1080, 1366x768, 1024x768, 640x480, 375x812</v>
       </c>
-      <c r="I50" t="str" xml:space="preserve">
+      <c r="I61" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Iterate through viewports
 2. Verify H1 visible
 3. Check document scrollWidth &lt;= clientWidth</v>
       </c>
-      <c r="J50" t="str">
+      <c r="J61" t="str">
         <v>No unwanted horizontal scrollbars; layout scales fluidly</v>
       </c>
-      <c r="K50" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="51" xml:space="preserve">
-      <c r="A51" t="str">
+      <c r="K61" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="62" xml:space="preserve">
+      <c r="A62" t="str">
         <v>TC-LOC-01</v>
       </c>
-      <c r="B51" t="str">
+      <c r="B62" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C51" t="str">
+      <c r="C62" t="str">
         <v>Localization &amp; RTL</v>
       </c>
-      <c r="D51" t="str">
+      <c r="D62" t="str">
         <v>Localization &amp; Arabic RTL Layout Suite</v>
       </c>
-      <c r="E51" t="str">
+      <c r="E62" t="str">
         <v>tests/05-arabic-rtl-localization.spec.ts</v>
       </c>
-      <c r="F51" t="str">
+      <c r="F62" t="str">
         <v>Positive / i18n</v>
       </c>
-      <c r="G51" t="str">
+      <c r="G62" t="str">
         <v>Language translation widget and default language settings</v>
       </c>
-      <c r="H51" t="str">
+      <c r="H62" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I51" t="str" xml:space="preserve">
+      <c r="I62" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open language dropdown
 2. Verify English, Arabic, French options available</v>
       </c>
-      <c r="J51" t="str">
+      <c r="J62" t="str">
         <v>Language switcher provides multilingual selection</v>
       </c>
-      <c r="K51" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="52" xml:space="preserve">
-      <c r="A52" t="str">
+      <c r="K62" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="63" xml:space="preserve">
+      <c r="A63" t="str">
         <v>TC-LOC-02</v>
       </c>
-      <c r="B52" t="str">
+      <c r="B63" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C52" t="str">
+      <c r="C63" t="str">
         <v>Localization &amp; RTL</v>
       </c>
-      <c r="D52" t="str">
+      <c r="D63" t="str">
         <v>Localization &amp; Arabic RTL Layout Suite</v>
       </c>
-      <c r="E52" t="str">
+      <c r="E63" t="str">
         <v>tests/05-arabic-rtl-localization.spec.ts</v>
       </c>
-      <c r="F52" t="str">
+      <c r="F63" t="str">
         <v>Positive / Currency</v>
       </c>
-      <c r="G52" t="str">
+      <c r="G63" t="str">
         <v>Algerian Dinar (DZD) currency formatting across components</v>
       </c>
-      <c r="H52" t="str">
+      <c r="H63" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I52" t="str" xml:space="preserve">
+      <c r="I63" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Inspect currency button
 2. Check DZD / دج designation in pricing displays</v>
       </c>
-      <c r="J52" t="str">
+      <c r="J63" t="str">
         <v>Default currency is Algerian Dinar (DZD)</v>
       </c>
-      <c r="K52" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="53" xml:space="preserve">
-      <c r="A53" t="str">
+      <c r="K63" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="64" xml:space="preserve">
+      <c r="A64" t="str">
         <v>TC-LOC-03</v>
       </c>
-      <c r="B53" t="str">
+      <c r="B64" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C53" t="str">
+      <c r="C64" t="str">
         <v>Localization &amp; RTL</v>
       </c>
-      <c r="D53" t="str">
+      <c r="D64" t="str">
         <v>Localization &amp; Arabic RTL Layout Suite</v>
       </c>
-      <c r="E53" t="str">
+      <c r="E64" t="str">
         <v>tests/05-arabic-rtl-localization.spec.ts</v>
       </c>
-      <c r="F53" t="str">
+      <c r="F64" t="str">
         <v>Positive / Legal Info</v>
       </c>
-      <c r="G53" t="str">
+      <c r="G64" t="str">
         <v>Algerian legal entity, local address and contact in footer</v>
       </c>
-      <c r="H53" t="str">
+      <c r="H64" t="str">
         <v>Homepage footer visible</v>
       </c>
-      <c r="I53" t="str" xml:space="preserve">
+      <c r="I64" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Inspect footer address
 2. Check SARL BILLETIX ALGERIE TRAVEL, Hai Khemisti, Oran</v>
       </c>
-      <c r="J53" t="str">
+      <c r="J64" t="str">
         <v>Local Algerian commercial entity registration confirmed in footer</v>
       </c>
-      <c r="K53" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="54" xml:space="preserve">
-      <c r="A54" t="str">
+      <c r="K64" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="65" xml:space="preserve">
+      <c r="A65" t="str">
         <v>TC-LOC-04</v>
       </c>
-      <c r="B54" t="str">
+      <c r="B65" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C54" t="str">
+      <c r="C65" t="str">
         <v>Localization &amp; RTL</v>
       </c>
-      <c r="D54" t="str">
+      <c r="D65" t="str">
         <v>Localization &amp; Arabic RTL Layout Suite</v>
       </c>
-      <c r="E54" t="str">
+      <c r="E65" t="str">
         <v>tests/05-arabic-rtl-localization.spec.ts</v>
       </c>
-      <c r="F54" t="str">
+      <c r="F65" t="str">
         <v>Positive / Trust Badges</v>
       </c>
-      <c r="G54" t="str">
+      <c r="G65" t="str">
         <v>Legal compliance badges (IATA, PCI-DSS, Authorized agent)</v>
       </c>
-      <c r="H54" t="str">
+      <c r="H65" t="str">
         <v>Homepage footer visible</v>
       </c>
-      <c r="I54" t="str" xml:space="preserve">
+      <c r="I65" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Inspect security badges in footer
 2. Verify IATA accredited agent, PCI-DSS, and Card payment logos</v>
       </c>
-      <c r="J54" t="str">
+      <c r="J65" t="str">
         <v>Industry certification and accreditation badges clearly displayed</v>
       </c>
-      <c r="K54" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="55" xml:space="preserve">
-      <c r="A55" t="str">
+      <c r="K65" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="66" xml:space="preserve">
+      <c r="A66" t="str">
         <v>TC-A11Y-01</v>
       </c>
-      <c r="B55" t="str">
+      <c r="B66" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C55" t="str">
+      <c r="C66" t="str">
         <v>Accessibility (a11y)</v>
       </c>
-      <c r="D55" t="str">
+      <c r="D66" t="str">
         <v>Automated Accessibility Audit Suite</v>
       </c>
-      <c r="E55" t="str">
+      <c r="E66" t="str">
         <v>tests/06-accessibility-audit.spec.ts</v>
       </c>
-      <c r="F55" t="str">
+      <c r="F66" t="str">
         <v>A11y / Axe-Core</v>
       </c>
-      <c r="G55" t="str">
+      <c r="G66" t="str">
         <v>Scan homepage for WCAG 2.1 Level A &amp; AA violations</v>
       </c>
-      <c r="H55" t="str">
+      <c r="H66" t="str">
         <v>AxeBuilder injected onto homepage</v>
       </c>
-      <c r="I55" t="str" xml:space="preserve">
+      <c r="I66" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Run axe-core automated scanner
 2. Evaluate WCAG 2.1 Level A and AA violations</v>
       </c>
-      <c r="J55" t="str">
+      <c r="J66" t="str">
         <v>Automated scan produces structured accessibility report</v>
       </c>
-      <c r="K55" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="56" xml:space="preserve">
-      <c r="A56" t="str">
+      <c r="K66" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="67" xml:space="preserve">
+      <c r="A67" t="str">
         <v>TC-A11Y-02</v>
       </c>
-      <c r="B56" t="str">
+      <c r="B67" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C56" t="str">
+      <c r="C67" t="str">
         <v>Accessibility (a11y)</v>
       </c>
-      <c r="D56" t="str">
+      <c r="D67" t="str">
         <v>Automated Accessibility Audit Suite</v>
       </c>
-      <c r="E56" t="str">
+      <c r="E67" t="str">
         <v>tests/06-accessibility-audit.spec.ts</v>
       </c>
-      <c r="F56" t="str">
+      <c r="F67" t="str">
         <v>A11y / Alt Text</v>
       </c>
-      <c r="G56" t="str">
+      <c r="G67" t="str">
         <v>Verify image elements have descriptive alternative text</v>
       </c>
-      <c r="H56" t="str">
+      <c r="H67" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I56" t="str" xml:space="preserve">
+      <c r="I67" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Query all &lt;img&gt; elements
 2. Verify presence of alt attribute</v>
       </c>
-      <c r="J56" t="str">
+      <c r="J67" t="str">
         <v>Images contain alt text for screen-reader accessibility</v>
       </c>
-      <c r="K56" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="57" xml:space="preserve">
-      <c r="A57" t="str">
+      <c r="K67" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="68" xml:space="preserve">
+      <c r="A68" t="str">
         <v>TC-A11Y-03</v>
       </c>
-      <c r="B57" t="str">
+      <c r="B68" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C57" t="str">
+      <c r="C68" t="str">
         <v>Accessibility (a11y)</v>
       </c>
-      <c r="D57" t="str">
+      <c r="D68" t="str">
         <v>Automated Accessibility Audit Suite</v>
       </c>
-      <c r="E57" t="str">
+      <c r="E68" t="str">
         <v>tests/06-accessibility-audit.spec.ts</v>
       </c>
-      <c r="F57" t="str">
+      <c r="F68" t="str">
         <v>A11y / ARIA</v>
       </c>
-      <c r="G57" t="str">
+      <c r="G68" t="str">
         <v>Verify interactive search button has accessible name</v>
       </c>
-      <c r="H57" t="str">
+      <c r="H68" t="str">
         <v>Homepage loaded</v>
       </c>
-      <c r="I57" t="str" xml:space="preserve">
+      <c r="I68" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Locate primary flight search button
 2. Check accessible name via getByRole("button", { name: ... })</v>
       </c>
-      <c r="J57" t="str">
+      <c r="J68" t="str">
         <v>Primary CTA has clear accessible name for assistive technologies</v>
       </c>
-      <c r="K57" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="58" xml:space="preserve">
-      <c r="A58" t="str">
+      <c r="K68" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="69" xml:space="preserve">
+      <c r="A69" t="str">
         <v>TC-SUP-01</v>
       </c>
-      <c r="B58" t="str">
+      <c r="B69" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C58" t="str">
+      <c r="C69" t="str">
         <v>Support &amp; Policies</v>
       </c>
-      <c r="D58" t="str">
+      <c r="D69" t="str">
         <v>Customer Support, FAQ &amp; Legal Policies Suite</v>
       </c>
-      <c r="E58" t="str">
+      <c r="E69" t="str">
         <v>tests/08-support-and-policies.spec.ts</v>
       </c>
-      <c r="F58" t="str">
+      <c r="F69" t="str">
         <v>Positive / Support</v>
       </c>
-      <c r="G58" t="str">
+      <c r="G69" t="str">
         <v>Contact Us page elements and official contact channels</v>
       </c>
-      <c r="H58" t="str">
+      <c r="H69" t="str">
         <v>Navigation to /support/contact</v>
       </c>
-      <c r="I58" t="str" xml:space="preserve">
+      <c r="I69" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Load support page
 2. Verify phone number, email address, and office location are displayed</v>
       </c>
-      <c r="J58" t="str">
+      <c r="J69" t="str">
         <v>Official customer support channels are clearly listed</v>
       </c>
-      <c r="K58" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="59" xml:space="preserve">
-      <c r="A59" t="str">
+      <c r="K69" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="70" xml:space="preserve">
+      <c r="A70" t="str">
         <v>TC-SUP-02</v>
       </c>
-      <c r="B59" t="str">
+      <c r="B70" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C59" t="str">
+      <c r="C70" t="str">
         <v>Support &amp; Policies</v>
       </c>
-      <c r="D59" t="str">
+      <c r="D70" t="str">
         <v>Customer Support, FAQ &amp; Legal Policies Suite</v>
       </c>
-      <c r="E59" t="str">
+      <c r="E70" t="str">
         <v>tests/08-support-and-policies.spec.ts</v>
       </c>
-      <c r="F59" t="str">
+      <c r="F70" t="str">
         <v>Negative / Form</v>
       </c>
-      <c r="G59" t="str">
+      <c r="G70" t="str">
         <v>Contact Us form invalid input validation</v>
       </c>
-      <c r="H59" t="str">
+      <c r="H70" t="str">
         <v>Contact form loaded</v>
       </c>
-      <c r="I59" t="str" xml:space="preserve">
+      <c r="I70" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Submit empty or malformed contact message
 2. Check validation response</v>
       </c>
-      <c r="J59" t="str">
+      <c r="J70" t="str">
         <v>Form highlights missing fields or displays validation warning</v>
       </c>
-      <c r="K59" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="60" xml:space="preserve">
-      <c r="A60" t="str">
+      <c r="K70" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="71" xml:space="preserve">
+      <c r="A71" t="str">
         <v>TC-SUP-03</v>
       </c>
-      <c r="B60" t="str">
+      <c r="B71" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C60" t="str">
+      <c r="C71" t="str">
         <v>Support &amp; Policies</v>
       </c>
-      <c r="D60" t="str">
+      <c r="D71" t="str">
         <v>Customer Support, FAQ &amp; Legal Policies Suite</v>
       </c>
-      <c r="E60" t="str">
+      <c r="E71" t="str">
         <v>tests/08-support-and-policies.spec.ts</v>
       </c>
-      <c r="F60" t="str">
+      <c r="F71" t="str">
         <v>Positive / Accordion</v>
       </c>
-      <c r="G60" t="str">
+      <c r="G71" t="str">
         <v>FAQ page accordion questions and answer expansion</v>
       </c>
-      <c r="H60" t="str">
+      <c r="H71" t="str">
         <v>Navigation to /faq</v>
       </c>
-      <c r="I60" t="str" xml:space="preserve">
+      <c r="I71" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Locate FAQ accordion headers
 2. Click question item
 3. Verify answer body expands</v>
       </c>
-      <c r="J60" t="str">
+      <c r="J71" t="str">
         <v>FAQ accordion expands to reveal detailed answer text upon interaction</v>
       </c>
-      <c r="K60" t="str">
-        <v>Passed</v>
-      </c>
-    </row>
-    <row r="61" xml:space="preserve">
-      <c r="A61" t="str">
+      <c r="K71" t="str">
+        <v>Passed</v>
+      </c>
+    </row>
+    <row r="72" xml:space="preserve">
+      <c r="A72" t="str">
         <v>TC-SUP-04</v>
       </c>
-      <c r="B61" t="str">
+      <c r="B72" t="str">
         <v>Day 1</v>
       </c>
-      <c r="C61" t="str">
+      <c r="C72" t="str">
         <v>Support &amp; Policies</v>
       </c>
-      <c r="D61" t="str">
+      <c r="D72" t="str">
         <v>Customer Support, FAQ &amp; Legal Policies Suite</v>
       </c>
-      <c r="E61" t="str">
+      <c r="E72" t="str">
         <v>tests/08-support-and-policies.spec.ts</v>
       </c>
-      <c r="F61" t="str">
+      <c r="F72" t="str">
         <v>Positive / Legal Integrity</v>
       </c>
-      <c r="G61" t="str">
+      <c r="G72" t="str">
         <v>Legal policy pages integrity (Terms &amp; Conditions, Privacy, Refund)</v>
       </c>
-      <c r="H61" t="str">
+      <c r="H72" t="str">
         <v>Navigation to legal policy routes</v>
       </c>
-      <c r="I61" t="str" xml:space="preserve">
+      <c r="I72" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Load /terms-conditions, /privacy-policy, /refund-policy
 2. Check HTTP status and H1 headings</v>
       </c>
-      <c r="J61" t="str">
+      <c r="J72" t="str">
         <v>All policy pages load cleanly with valid legal text and headings</v>
       </c>
-      <c r="K61" t="str">
+      <c r="K72" t="str">
         <v>Passed</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K72"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -2663,7 +3061,7 @@
         <v>Generated Date:</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-09-23</v>
+        <v>2026-09-29</v>
       </c>
     </row>
     <row r="3">
@@ -2701,13 +3099,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Day 3 (Checkout, Payment Mocking, PNR)</v>
+        <v>Day 4 (Security Fuzzing &amp; Performance Web Vitals)</v>
       </c>
       <c r="B7">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C7">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -2718,13 +3116,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Day 2 (Search Matrix, Filters, Auth &amp; Pax)</v>
+        <v>Day 3 (Checkout, Payment Mocking, PNR)</v>
       </c>
       <c r="B8">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C8">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -2735,13 +3133,13 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Day 1 (UI Baseline, Localization, A11y, Support)</v>
+        <v>Day 2 (Search Matrix, Filters, Auth &amp; Pax)</v>
       </c>
       <c r="B9">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C9">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -2750,26 +3148,43 @@
         <v>100%</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="str">
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Day 1 (UI Baseline, Localization, A11y, Support)</v>
+      </c>
+      <c r="B10">
+        <v>16</v>
+      </c>
+      <c r="C10">
+        <v>16</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10" t="str">
+        <v>100%</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>Total Suite</v>
       </c>
-      <c r="B11">
-        <v>60</v>
-      </c>
-      <c r="C11">
-        <v>60</v>
-      </c>
-      <c r="D11">
+      <c r="B12">
+        <v>71</v>
+      </c>
+      <c r="C12">
+        <v>71</v>
+      </c>
+      <c r="D12">
         <v>0</v>
       </c>
-      <c r="E11" t="str">
+      <c r="E12" t="str">
         <v>100%</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>